<commit_message>
Add configurable volunteer records and connected event workspaces
</commit_message>
<xml_diff>
--- a/artifacts/exports/shuori-demo-project-plan.xlsx
+++ b/artifacts/exports/shuori-demo-project-plan.xlsx
@@ -38,7 +38,7 @@
     <t>守織 SHUORI · Workbook overview</t>
   </si>
   <si>
-    <t>Generated 2026-10-08 10:10:35 JST · Asia/Tokyo · demo · version 1.2.0</t>
+    <t>Generated 2026-10-08 17:07:03 JST · Asia/Tokyo · demo · version 1.3.0</t>
   </si>
   <si>
     <t>project-plan | All records in the stated scope | Project: project-welcome | View label: Complete plan | tasks &amp; critical path</t>
@@ -1561,10 +1561,10 @@
         <v>1</v>
       </c>
       <c r="P6" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="Q6" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
   </sheetData>
@@ -1807,10 +1807,10 @@
         <v>1</v>
       </c>
       <c r="R6" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="S6" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -1866,10 +1866,10 @@
         <v>1</v>
       </c>
       <c r="R7" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="S7" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -1925,10 +1925,10 @@
         <v>1</v>
       </c>
       <c r="R8" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="S8" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -1984,10 +1984,10 @@
         <v>1</v>
       </c>
       <c r="R9" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="S9" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -2043,10 +2043,10 @@
         <v>1</v>
       </c>
       <c r="R10" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="S10" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -2102,10 +2102,10 @@
         <v>1</v>
       </c>
       <c r="R11" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="S11" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
   </sheetData>
@@ -2529,10 +2529,10 @@
         <v>1</v>
       </c>
       <c r="S6" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T6" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -2591,10 +2591,10 @@
         <v>1</v>
       </c>
       <c r="S7" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T7" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -2653,10 +2653,10 @@
         <v>1</v>
       </c>
       <c r="S8" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T8" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -2715,10 +2715,10 @@
         <v>1</v>
       </c>
       <c r="S9" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T9" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -2777,10 +2777,10 @@
         <v>1</v>
       </c>
       <c r="S10" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T10" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -2839,10 +2839,10 @@
         <v>1</v>
       </c>
       <c r="S11" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T11" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="12" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -2901,10 +2901,10 @@
         <v>1</v>
       </c>
       <c r="S12" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T12" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -2963,10 +2963,10 @@
         <v>1</v>
       </c>
       <c r="S13" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T13" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="14" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -3025,10 +3025,10 @@
         <v>1</v>
       </c>
       <c r="S14" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T14" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -3087,10 +3087,10 @@
         <v>1</v>
       </c>
       <c r="S15" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T15" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="16" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -3149,10 +3149,10 @@
         <v>1</v>
       </c>
       <c r="S16" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T16" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="17" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -3211,10 +3211,10 @@
         <v>1</v>
       </c>
       <c r="S17" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T17" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="18" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -3273,10 +3273,10 @@
         <v>1</v>
       </c>
       <c r="S18" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T18" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="19" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -3335,10 +3335,10 @@
         <v>1</v>
       </c>
       <c r="S19" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T19" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="20" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -3397,10 +3397,10 @@
         <v>1</v>
       </c>
       <c r="S20" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T20" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="21" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -3459,10 +3459,10 @@
         <v>1</v>
       </c>
       <c r="S21" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T21" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -3521,10 +3521,10 @@
         <v>1</v>
       </c>
       <c r="S22" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T22" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="23" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -3583,10 +3583,10 @@
         <v>1</v>
       </c>
       <c r="S23" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T23" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="24" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -3645,10 +3645,10 @@
         <v>1</v>
       </c>
       <c r="S24" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T24" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="25" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -3707,10 +3707,10 @@
         <v>1</v>
       </c>
       <c r="S25" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T25" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="26" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -3769,10 +3769,10 @@
         <v>1</v>
       </c>
       <c r="S26" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T26" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="27" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -3831,10 +3831,10 @@
         <v>1</v>
       </c>
       <c r="S27" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T27" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="28" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -3893,10 +3893,10 @@
         <v>1</v>
       </c>
       <c r="S28" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T28" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="29" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -3955,10 +3955,10 @@
         <v>1</v>
       </c>
       <c r="S29" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T29" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="30" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -4017,10 +4017,10 @@
         <v>1</v>
       </c>
       <c r="S30" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T30" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="31" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -4079,10 +4079,10 @@
         <v>1</v>
       </c>
       <c r="S31" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T31" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="32" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -4141,10 +4141,10 @@
         <v>1</v>
       </c>
       <c r="S32" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T32" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="33" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -4203,10 +4203,10 @@
         <v>1</v>
       </c>
       <c r="S33" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T33" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="34" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -4265,10 +4265,10 @@
         <v>1</v>
       </c>
       <c r="S34" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T34" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="35" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -4327,10 +4327,10 @@
         <v>1</v>
       </c>
       <c r="S35" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T35" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="36" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -4389,10 +4389,10 @@
         <v>1</v>
       </c>
       <c r="S36" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T36" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="37" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -4451,10 +4451,10 @@
         <v>1</v>
       </c>
       <c r="S37" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T37" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="38" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -4513,10 +4513,10 @@
         <v>1</v>
       </c>
       <c r="S38" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T38" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="39" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -4575,10 +4575,10 @@
         <v>1</v>
       </c>
       <c r="S39" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T39" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="40" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -4637,10 +4637,10 @@
         <v>1</v>
       </c>
       <c r="S40" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T40" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="41" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -4699,10 +4699,10 @@
         <v>1</v>
       </c>
       <c r="S41" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T41" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="42" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -4761,10 +4761,10 @@
         <v>1</v>
       </c>
       <c r="S42" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T42" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="43" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -4823,10 +4823,10 @@
         <v>1</v>
       </c>
       <c r="S43" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T43" s="15">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
     <row r="44" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -4885,10 +4885,10 @@
         <v>1</v>
       </c>
       <c r="S44" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
       <c r="T44" s="12">
-        <v>46303.35549128472</v>
+        <v>46303.70653649306</v>
       </c>
     </row>
   </sheetData>

</xml_diff>